<commit_message>
fix(coords): correct Headland district to Chai Wan, unify multi-phase mobility and fix straight-line walking routes
</commit_message>
<xml_diff>
--- a/全港一手新盘空间区域与商圈归属重划表.xlsx
+++ b/全港一手新盘空间区域与商圈归属重划表.xlsx
@@ -9553,17 +9553,17 @@
       </c>
       <c r="C129" s="7" t="inlineStr">
         <is>
-          <t>港岛南区</t>
+          <t>港岛东区</t>
         </is>
       </c>
       <c r="D129" s="7" t="inlineStr">
         <is>
-          <t>石澳、大浪湾及鹤咀</t>
+          <t>柴湾及小西湾</t>
         </is>
       </c>
       <c r="E129" s="8" t="inlineStr">
         <is>
-          <t>Statutory Scheme (S/H20/25)</t>
+          <t>Chai Wan &amp; Siu Sai Wan</t>
         </is>
       </c>
       <c r="F129" s="8" t="inlineStr">

</xml_diff>